<commit_message>
feat(server): 回调事件 inbox、轮询兜底与 dead-letter 补偿
- P3-09 事件 inbox：Postgres payload AES-256-GCM 加密 + dedupeKey 幂等入库
- ticket 回调经 inbox 消费：appended→processed / 失败→dead（attempts+last_error）
- 双保险去重：nonce 防线失效时（跨重启），同一报文重发按内容判重不重复消费
- replayTicketDeadLetter：dead-letter 人工重放，非法 payload 保持 dead
- 对账服务：ticket 新鲜度巡检（15 分钟阈值告警）+ api_get_authorizer_list 轮询恢复丢回调的 unauthorized（本地 active 远端移除→标记 revoked）
- 路由：/wechat/reconciliation、/wechat/inbox/dead、POST /wechat/inbox/replay（operator/admin）
- @gravitas/server 0.1.11 → 0.1.12
</commit_message>
<xml_diff>
--- a/.context/plan/new-media-p0-p4-task-ledger.xlsx
+++ b/.context/plan/new-media-p0-p4-task-ledger.xlsx
@@ -2744,7 +2744,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>待开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2762,12 +2762,12 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>事件 inbox、幂等消费、dead-letter</t>
+          <t>事件 inbox（Postgres payload 加密 + dedupeKey 幂等入库）、ticket 经 inbox 消费（processed/dead 状态机）、dead-letter 人工重放（replayTicketDeadLetter）、ticket 新鲜度巡检与授权账号对账（轮询恢复丢回调的 unauthorized）</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>重复回调不重复执行；丢回调可由轮询恢复；失败可人工重放</t>
+          <t>重复回调不重复执行：nonce 防线 + inbox 内容判重双保险，跨重启同报文重发最多消费一次；丢回调可恢复：ticket 过期告警 + api_get_authorizer_list 对账把本地 active 远端已移除的账号标记 revoked；失败可人工重放：/wechat/inbox/dead 列出、/wechat/inbox/replay 重放</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">

</xml_diff>